<commit_message>
updated literature with new referneces
</commit_message>
<xml_diff>
--- a/0-complete_literature_data/analysis_single_vs_multi_and_impreg_inside.xlsx
+++ b/0-complete_literature_data/analysis_single_vs_multi_and_impreg_inside.xlsx
@@ -476,13 +476,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="C3" t="n">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="D3" t="n">
-        <v>1.621</v>
+        <v>1.608</v>
       </c>
     </row>
     <row r="4">
@@ -492,13 +492,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>349</v>
-      </c>
-      <c r="C4" t="n">
-        <v>212</v>
-      </c>
+        <v>353</v>
+      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="n">
-        <v>1.646</v>
+        <v>1.634</v>
       </c>
     </row>
   </sheetData>
@@ -542,7 +540,7 @@
         <v>19</v>
       </c>
       <c r="C2" t="n">
-        <v>57.6</v>
+        <v>55.9</v>
       </c>
     </row>
     <row r="3">
@@ -552,10 +550,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C3" t="n">
-        <v>42.4</v>
+        <v>44.1</v>
       </c>
     </row>
   </sheetData>
@@ -569,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -596,10 +594,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C2" t="n">
-        <v>54.1</v>
+        <v>55.7</v>
       </c>
     </row>
     <row r="3">
@@ -618,7 +616,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>One-pot / in-situ encapsulation</t>
+          <t>Chemical vapor deposition / infiltration</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -631,7 +629,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Chemical vapor deposition / infiltration</t>
+          <t>One-pot / in-situ encapsulation</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -651,19 +649,6 @@
         <v>1</v>
       </c>
       <c r="C6" t="n">
-        <v>1.6</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Others</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" t="n">
         <v>1.6</v>
       </c>
     </row>
@@ -678,7 +663,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N34"/>
+  <dimension ref="A1:N35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1048,7 +1033,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1104,7 +1089,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1160,7 +1145,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1218,7 +1203,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1276,7 +1261,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1334,7 +1319,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1392,7 +1377,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1452,7 +1437,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1512,7 +1497,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1568,7 +1553,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1624,7 +1609,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -1680,7 +1665,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -1736,7 +1721,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -1796,7 +1781,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -1848,15 +1833,15 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Pt</t>
+          <t>Pd</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>MIL-101(Cr)</t>
+          <t>UiO-66-NH2</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1869,11 +1854,11 @@
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="n">
-        <v>42</v>
+        <v>241</v>
       </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="n">
-        <v>42</v>
+        <v>241</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
@@ -1882,7 +1867,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>['Pt']</t>
+          <t>['Pd']</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -1908,11 +1893,11 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Zr6(μ3-O)4(μ3-OH)4(bpdc)5.94(L1)0.06 (UiO-67-1)</t>
+          <t>MIL-101(Cr)</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -1920,24 +1905,16 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The [Ir(ppy)2(bpy)]Cl-derived dicarboxylic acids H2L1 was synthesized by treating [Ir(ppy)2Cl]2 with diethyl (2,2′-bipyridine)-5,5′-dicarboxylate (Et2L1) </t>
-        </is>
-      </c>
+          <t>DSM</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
       <c r="G22" t="n">
-        <v>55</v>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>汪老师的文章，从TEM图判断为0</t>
-        </is>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="H22" t="inlineStr"/>
       <c r="I22" t="n">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
@@ -1956,7 +1933,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>Solution impregnation</t>
+          <t>Double solvent method</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -1972,11 +1949,11 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Zr6(μ3-O)4(μ3-OH)4(L2)6·64DMF (UiO-67-2)</t>
+          <t>Zr6(μ3-O)4(μ3-OH)4(bpdc)5.94(L1)0.06 (UiO-67-1)</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -1989,7 +1966,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>The [Ir(ppy)2(bpy)]Cl-derived dicarboxylic acids  H2L2 was synthesized by treating [Ir(ppy)2Cl]2 with dimethyl (2,2′-bipyridine)-5,5′-dibenzoate (Me2L2)</t>
+          <t xml:space="preserve">The [Ir(ppy)2(bpy)]Cl-derived dicarboxylic acids H2L1 was synthesized by treating [Ir(ppy)2Cl]2 with diethyl (2,2′-bipyridine)-5,5′-dicarboxylate (Et2L1) </t>
         </is>
       </c>
       <c r="G23" t="n">
@@ -2036,11 +2013,11 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>MIL-101(Cr)</t>
+          <t>Zr6(μ3-O)4(μ3-OH)4(L2)6·64DMF (UiO-67-2)</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -2048,20 +2025,24 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>DSM</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>The [Ir(ppy)2(bpy)]Cl-derived dicarboxylic acids  H2L2 was synthesized by treating [Ir(ppy)2Cl]2 with dimethyl (2,2′-bipyridine)-5,5′-dibenzoate (Me2L2)</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>64</v>
-      </c>
-      <c r="H24" t="inlineStr"/>
+        <v>55</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>汪老师的文章，从TEM图判断为0</t>
+        </is>
+      </c>
       <c r="I24" t="n">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
@@ -2080,7 +2061,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>Double solvent method</t>
+          <t>Solution impregnation</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2096,11 +2077,11 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>UiO-66-NH2(Zr)</t>
+          <t>MIL-101(Cr)</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -2108,16 +2089,20 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr"/>
+          <t>DSM</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
       <c r="G25" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
@@ -2136,7 +2121,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Solution impregnation</t>
+          <t>Double solvent method</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -2152,11 +2137,11 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>240</v>
+        <v>194</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>UiO-66</t>
+          <t>UiO-66-NH2(Zr)</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -2169,11 +2154,11 @@
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="n">
-        <v>216</v>
+        <v>65</v>
       </c>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="n">
-        <v>216</v>
+        <v>65</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
@@ -2208,11 +2193,11 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>MIL-101</t>
+          <t>UiO-66</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -2220,16 +2205,16 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>DSM</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="n">
-        <v>126</v>
+        <v>216</v>
       </c>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="n">
-        <v>126</v>
+        <v>216</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
@@ -2248,7 +2233,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>Double solvent method</t>
+          <t>Solution impregnation</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2260,15 +2245,15 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Rh</t>
+          <t>Pt</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ZIF-8(Zn)</t>
+          <t>MIL-101</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -2276,20 +2261,16 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Before Reaction</t>
-        </is>
-      </c>
+          <t>DSM</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
       <c r="G28" t="n">
-        <v>66</v>
+        <v>126</v>
       </c>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="n">
-        <v>66</v>
+        <v>126</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
@@ -2298,7 +2279,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>['Rh']</t>
+          <t>['Pt']</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -2308,7 +2289,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>Solution impregnation</t>
+          <t>Double solvent method</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2320,15 +2301,15 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Cu</t>
+          <t>Rh</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>NU-1000-NH2/PrSH(Zr)</t>
+          <t>ZIF-8(Zn)</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -2339,13 +2320,17 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Before Reaction</t>
+        </is>
+      </c>
       <c r="G29" t="n">
-        <v>193</v>
+        <v>66</v>
       </c>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="n">
-        <v>193</v>
+        <v>66</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
@@ -2354,7 +2339,7 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>['Cu']</t>
+          <t>['Rh']</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
@@ -2380,11 +2365,11 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>UiO-66-NH2</t>
+          <t>NU-1000-NH2/PrSH(Zr)</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -2397,11 +2382,11 @@
       </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="n">
-        <v>204</v>
+        <v>193</v>
       </c>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="n">
-        <v>204</v>
+        <v>193</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
@@ -2436,11 +2421,11 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>MOF-801</t>
+          <t>UiO-66-NH2</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -2492,11 +2477,11 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2Bn@UiO-67</t>
+          <t>MOF-801</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -2509,11 +2494,11 @@
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="n">
-        <v>218</v>
+        <v>204</v>
       </c>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="n">
-        <v>218</v>
+        <v>204</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
@@ -2548,11 +2533,11 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>NU-1000-NH2</t>
+          <t>2Bn@UiO-67</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -2565,11 +2550,11 @@
       </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="n">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="n">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
@@ -2600,15 +2585,15 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Ni</t>
+          <t>Cu</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>276</v>
+        <v>268</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>UiO-66</t>
+          <t>NU-1000-NH2</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -2621,33 +2606,89 @@
       </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="n">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="n">
+        <v>225</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Single-metal</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>['Cu']</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Inside</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Solution impregnation</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>Liquid-phase impregnation</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Ni</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>280</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>UiO-66</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="n">
         <v>220</v>
       </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>Single-metal</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr">
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="n">
+        <v>220</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Single-metal</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
         <is>
           <t>['Ni']</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>Inside</t>
-        </is>
-      </c>
-      <c r="M34" t="inlineStr">
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Inside</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
         <is>
           <t>Solution impregnation</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr">
+      <c r="N35" t="inlineStr">
         <is>
           <t>Liquid-phase impregnation</t>
         </is>

</xml_diff>